<commit_message>
October 2026 update: GPU rates, gateway fees, new gateways, competitor churn
- Capacity: on-demand $4.50 and reserved $3.05 per GPU-hour as market
  placeholders (H100 prices up ~15% in a year; 1-year deals ~32% off).
- Gateways: Vercel and OpenRouter fee 0% (they list Jev at the direct
  price); DigitalOcean marked unconfirmed; Netlify and Cloudflare added.
- Free credit: gateway-funded credit is never TypeSafe's grant.
- Forecast: competitor_churn input (low case 3%/month on self-serve) in
  Excel and the Python mirror; parity test still passes.
- LOGIC_REVIEW assumptions 4, 8 and 14 updated; agent routing keywords.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PxrWEnqjAJujA3Cx9ACajN
</commit_message>
<xml_diff>
--- a/template/Jev_Close_Template.xlsx
+++ b/template/Jev_Close_Template.xlsx
@@ -939,7 +939,7 @@
         <v/>
       </c>
       <c r="F8" s="13">
-        <f>Overrides!$E$22</f>
+        <f>Overrides!$E$25</f>
         <v/>
       </c>
     </row>
@@ -9077,7 +9077,7 @@
         </is>
       </c>
       <c r="B6" s="43">
-        <f>Overrides!$E$23</f>
+        <f>Overrides!$E$26</f>
         <v/>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -9093,7 +9093,7 @@
         </is>
       </c>
       <c r="B7" s="37">
-        <f>Overrides!$E$24</f>
+        <f>Overrides!$E$27</f>
         <v/>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -9109,12 +9109,12 @@
         </is>
       </c>
       <c r="B8" s="14">
-        <f>Overrides!$E$25</f>
+        <f>Overrides!$E$28</f>
         <v/>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>From your capacity contract.</t>
+          <t>Market placeholder (Oct 2026, ~32% below on-demand). Replace with the contracted rate.</t>
         </is>
       </c>
     </row>
@@ -9125,12 +9125,12 @@
         </is>
       </c>
       <c r="B9" s="14">
-        <f>Overrides!$E$26</f>
+        <f>Overrides!$E$29</f>
         <v/>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Same provider tier.</t>
+          <t>Market placeholder (Oct 2026): H100 at specialist GPU clouds. Same provider tier as reserved.</t>
         </is>
       </c>
     </row>
@@ -9141,7 +9141,7 @@
         </is>
       </c>
       <c r="B10" s="34">
-        <f>Overrides!$E$27</f>
+        <f>Overrides!$E$30</f>
         <v/>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -9157,7 +9157,7 @@
         </is>
       </c>
       <c r="B11" s="34">
-        <f>Overrides!$E$28</f>
+        <f>Overrides!$E$31</f>
         <v/>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -10083,29 +10083,29 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>signup_growth.low</t>
+          <t>competitor_churn.low</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Forecast: new signups monthly growth, low</t>
-        </is>
-      </c>
-      <c r="C17" s="25" t="n">
-        <v>0</v>
+          <t>Forecast: Self-serve tokens lost to competitors, per month, low</t>
+        </is>
+      </c>
+      <c r="C17" s="50" t="n">
+        <v>0.03</v>
       </c>
       <c r="D17" s="51" t="n"/>
       <c r="E17" s="27">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D17),D17&gt;=-0.5,D17&lt;=1),D17,C17),C17)</f>
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D17),D17&gt;=0,D17&lt;=0.5),D17,C17),C17)</f>
         <v/>
       </c>
       <c r="F17" s="3">
-        <f>IFERROR(IF(ISBLANK(D17),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D17),"Ignored: error value",IF(NOT(ISNUMBER(D17)),"Ignored: not a number",IF(OR(D17&lt;-0.5,D17&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D17),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D17),"Ignored: error value",IF(NOT(ISNUMBER(D17)),"Ignored: not a number",IF(OR(D17&lt;0,D17&gt;0.5),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>-0.5 to 1</t>
+          <t>0 to 0.5</t>
         </is>
       </c>
       <c r="H17" s="18" t="n"/>
@@ -10113,29 +10113,29 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>gateway_growth_decay</t>
+          <t>competitor_churn.base</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Forecast: gateway growth decay (base)</t>
-        </is>
-      </c>
-      <c r="C18" s="47" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D18" s="48" t="n"/>
-      <c r="E18" s="49">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D18),D18&gt;=0,D18&lt;=2),D18,C18),C18)</f>
+          <t>Forecast: Self-serve tokens lost to competitors, per month, base</t>
+        </is>
+      </c>
+      <c r="C18" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="51" t="n"/>
+      <c r="E18" s="27">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D18),D18&gt;=0,D18&lt;=0.5),D18,C18),C18)</f>
         <v/>
       </c>
       <c r="F18" s="3">
-        <f>IFERROR(IF(ISBLANK(D18),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D18),"Ignored: error value",IF(NOT(ISNUMBER(D18)),"Ignored: not a number",IF(OR(D18&lt;0,D18&gt;2),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D18),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D18),"Ignored: error value",IF(NOT(ISNUMBER(D18)),"Ignored: not a number",IF(OR(D18&lt;0,D18&gt;0.5),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>0 to 2</t>
+          <t>0 to 0.5</t>
         </is>
       </c>
       <c r="H18" s="18" t="n"/>
@@ -10143,29 +10143,29 @@
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>ent_ramp_days</t>
+          <t>competitor_churn.high</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Forecast: enterprise ramp length (days)</t>
-        </is>
-      </c>
-      <c r="C19" s="52" t="n">
-        <v>60</v>
-      </c>
-      <c r="D19" s="53" t="n"/>
-      <c r="E19" s="44">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D19),D19&gt;=1,D19&lt;=365),D19,C19),C19)</f>
+          <t>Forecast: Self-serve tokens lost to competitors, per month, high</t>
+        </is>
+      </c>
+      <c r="C19" s="50" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="51" t="n"/>
+      <c r="E19" s="27">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D19),D19&gt;=0,D19&lt;=0.5),D19,C19),C19)</f>
         <v/>
       </c>
       <c r="F19" s="3">
-        <f>IFERROR(IF(ISBLANK(D19),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D19),"Ignored: error value",IF(NOT(ISNUMBER(D19)),"Ignored: not a number",IF(OR(D19&lt;1,D19&gt;365),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D19),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D19),"Ignored: error value",IF(NOT(ISNUMBER(D19)),"Ignored: not a number",IF(OR(D19&lt;0,D19&gt;0.5),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>1 to 365</t>
+          <t>0 to 0.5</t>
         </is>
       </c>
       <c r="H19" s="18" t="n"/>
@@ -10173,30 +10173,29 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>price.self_serve</t>
+          <t>signup_growth.low</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Forecast: self-serve net $ per M tokens (price-change test)</t>
-        </is>
-      </c>
-      <c r="C20" s="26">
-        <f>IF(Monthly!M7=0,0,Monthly!M30/Monthly!M7)</f>
-        <v/>
-      </c>
-      <c r="D20" s="54" t="n"/>
-      <c r="E20" s="55">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D20),D20&gt;=0,D20&lt;=1),D20,C20),C20)</f>
+          <t>Forecast: new signups monthly growth, low</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="51" t="n"/>
+      <c r="E20" s="27">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D20),D20&gt;=-0.5,D20&lt;=1),D20,C20),C20)</f>
         <v/>
       </c>
       <c r="F20" s="3">
-        <f>IFERROR(IF(ISBLANK(D20),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D20),"Ignored: error value",IF(NOT(ISNUMBER(D20)),"Ignored: not a number",IF(OR(D20&lt;0,D20&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D20),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D20),"Ignored: error value",IF(NOT(ISNUMBER(D20)),"Ignored: not a number",IF(OR(D20&lt;-0.5,D20&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>-0.5 to 1</t>
         </is>
       </c>
       <c r="H20" s="18" t="n"/>
@@ -10204,30 +10203,29 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>price.gateway</t>
+          <t>gateway_growth_decay</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Forecast: gateway net $ per M tokens (price-change test)</t>
-        </is>
-      </c>
-      <c r="C21" s="26">
-        <f>IF(Monthly!M8=0,0,Monthly!M31/Monthly!M8)</f>
-        <v/>
-      </c>
-      <c r="D21" s="54" t="n"/>
-      <c r="E21" s="55">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D21),D21&gt;=0,D21&lt;=1),D21,C21),C21)</f>
+          <t>Forecast: gateway growth decay (base)</t>
+        </is>
+      </c>
+      <c r="C21" s="47" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D21" s="48" t="n"/>
+      <c r="E21" s="49">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D21),D21&gt;=0,D21&lt;=2),D21,C21),C21)</f>
         <v/>
       </c>
       <c r="F21" s="3">
-        <f>IFERROR(IF(ISBLANK(D21),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D21),"Ignored: error value",IF(NOT(ISNUMBER(D21)),"Ignored: not a number",IF(OR(D21&lt;0,D21&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D21),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D21),"Ignored: error value",IF(NOT(ISNUMBER(D21)),"Ignored: not a number",IF(OR(D21&lt;0,D21&gt;2),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>0 to 2</t>
         </is>
       </c>
       <c r="H21" s="18" t="n"/>
@@ -10235,30 +10233,29 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>price.list</t>
+          <t>ent_ramp_days</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Forecast: list $ per M tokens for pipeline deals</t>
-        </is>
-      </c>
-      <c r="C22" s="26">
-        <f>Data_Params!$B$4</f>
-        <v/>
-      </c>
-      <c r="D22" s="54" t="n"/>
-      <c r="E22" s="55">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D22),D22&gt;=0,D22&lt;=1),D22,C22),C22)</f>
+          <t>Forecast: enterprise ramp length (days)</t>
+        </is>
+      </c>
+      <c r="C22" s="52" t="n">
+        <v>60</v>
+      </c>
+      <c r="D22" s="53" t="n"/>
+      <c r="E22" s="44">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D22),D22&gt;=1,D22&lt;=365),D22,C22),C22)</f>
         <v/>
       </c>
       <c r="F22" s="3">
-        <f>IFERROR(IF(ISBLANK(D22),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D22),"Ignored: error value",IF(NOT(ISNUMBER(D22)),"Ignored: not a number",IF(OR(D22&lt;0,D22&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D22),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D22),"Ignored: error value",IF(NOT(ISNUMBER(D22)),"Ignored: not a number",IF(OR(D22&lt;1,D22&gt;365),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>0 to 1</t>
+          <t>1 to 365</t>
         </is>
       </c>
       <c r="H22" s="18" t="n"/>
@@ -10266,29 +10263,30 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>capacity.gpu_tokens_per_sec</t>
+          <t>price.self_serve</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Capacity: Tokens per second per busy GPU</t>
-        </is>
-      </c>
-      <c r="C23" s="52" t="n">
-        <v>20604</v>
-      </c>
-      <c r="D23" s="53" t="n"/>
-      <c r="E23" s="44">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D23),D23&gt;=1,D23&lt;=10000000),D23,C23),C23)</f>
+          <t>Forecast: self-serve net $ per M tokens (price-change test)</t>
+        </is>
+      </c>
+      <c r="C23" s="26">
+        <f>IF(Monthly!M7=0,0,Monthly!M30/Monthly!M7)</f>
+        <v/>
+      </c>
+      <c r="D23" s="54" t="n"/>
+      <c r="E23" s="55">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D23),D23&gt;=0,D23&lt;=1),D23,C23),C23)</f>
         <v/>
       </c>
       <c r="F23" s="3">
-        <f>IFERROR(IF(ISBLANK(D23),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D23),"Ignored: error value",IF(NOT(ISNUMBER(D23)),"Ignored: not a number",IF(OR(D23&lt;1,D23&gt;10000000),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D23),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D23),"Ignored: error value",IF(NOT(ISNUMBER(D23)),"Ignored: not a number",IF(OR(D23&lt;0,D23&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>1 to 1e+07</t>
+          <t>0 to 1</t>
         </is>
       </c>
       <c r="H23" s="18" t="n"/>
@@ -10296,29 +10294,30 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>capacity.peak_utilization</t>
+          <t>price.gateway</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Capacity: Target utilization at peak</t>
-        </is>
-      </c>
-      <c r="C24" s="50" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="D24" s="51" t="n"/>
-      <c r="E24" s="27">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D24),D24&gt;=0.05,D24&lt;=1),D24,C24),C24)</f>
+          <t>Forecast: gateway net $ per M tokens (price-change test)</t>
+        </is>
+      </c>
+      <c r="C24" s="26">
+        <f>IF(Monthly!M8=0,0,Monthly!M31/Monthly!M8)</f>
+        <v/>
+      </c>
+      <c r="D24" s="54" t="n"/>
+      <c r="E24" s="55">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D24),D24&gt;=0,D24&lt;=1),D24,C24),C24)</f>
         <v/>
       </c>
       <c r="F24" s="3">
-        <f>IFERROR(IF(ISBLANK(D24),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D24),"Ignored: error value",IF(NOT(ISNUMBER(D24)),"Ignored: not a number",IF(OR(D24&lt;0.05,D24&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D24),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D24),"Ignored: error value",IF(NOT(ISNUMBER(D24)),"Ignored: not a number",IF(OR(D24&lt;0,D24&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G24" s="7" t="inlineStr">
         <is>
-          <t>0.05 to 1</t>
+          <t>0 to 1</t>
         </is>
       </c>
       <c r="H24" s="18" t="n"/>
@@ -10326,29 +10325,30 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>capacity.reserved_rate</t>
+          <t>price.list</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>Capacity: Reserved rate ($ / GPU-hour)</t>
-        </is>
-      </c>
-      <c r="C25" s="56" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="D25" s="57" t="n"/>
-      <c r="E25" s="58">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D25),D25&gt;=0,D25&lt;=100),D25,C25),C25)</f>
+          <t>Forecast: list $ per M tokens for pipeline deals</t>
+        </is>
+      </c>
+      <c r="C25" s="26">
+        <f>Data_Params!$B$4</f>
+        <v/>
+      </c>
+      <c r="D25" s="54" t="n"/>
+      <c r="E25" s="55">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D25),D25&gt;=0,D25&lt;=1),D25,C25),C25)</f>
         <v/>
       </c>
       <c r="F25" s="3">
-        <f>IFERROR(IF(ISBLANK(D25),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D25),"Ignored: error value",IF(NOT(ISNUMBER(D25)),"Ignored: not a number",IF(OR(D25&lt;0,D25&gt;100),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D25),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D25),"Ignored: error value",IF(NOT(ISNUMBER(D25)),"Ignored: not a number",IF(OR(D25&lt;0,D25&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>0 to 100</t>
+          <t>0 to 1</t>
         </is>
       </c>
       <c r="H25" s="18" t="n"/>
@@ -10356,29 +10356,29 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>capacity.on_demand_rate</t>
+          <t>capacity.gpu_tokens_per_sec</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Capacity: On-demand rate ($ / GPU-hour)</t>
-        </is>
-      </c>
-      <c r="C26" s="56" t="n">
-        <v>3</v>
-      </c>
-      <c r="D26" s="57" t="n"/>
-      <c r="E26" s="58">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D26),D26&gt;=0,D26&lt;=100),D26,C26),C26)</f>
+          <t>Capacity: Tokens per second per busy GPU</t>
+        </is>
+      </c>
+      <c r="C26" s="52" t="n">
+        <v>20604</v>
+      </c>
+      <c r="D26" s="53" t="n"/>
+      <c r="E26" s="44">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D26),D26&gt;=1,D26&lt;=10000000),D26,C26),C26)</f>
         <v/>
       </c>
       <c r="F26" s="3">
-        <f>IFERROR(IF(ISBLANK(D26),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D26),"Ignored: error value",IF(NOT(ISNUMBER(D26)),"Ignored: not a number",IF(OR(D26&lt;0,D26&gt;100),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D26),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D26),"Ignored: error value",IF(NOT(ISNUMBER(D26)),"Ignored: not a number",IF(OR(D26&lt;1,D26&gt;10000000),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G26" s="7" t="inlineStr">
         <is>
-          <t>0 to 100</t>
+          <t>1 to 1e+07</t>
         </is>
       </c>
       <c r="H26" s="18" t="n"/>
@@ -10386,29 +10386,29 @@
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>capacity.peak_ratio_override</t>
+          <t>capacity.peak_utilization</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Capacity: Peak hour / average (override if no hourly data)</t>
-        </is>
-      </c>
-      <c r="C27" s="47" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="D27" s="48" t="n"/>
-      <c r="E27" s="49">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D27),D27&gt;=1,D27&lt;=20),D27,C27),C27)</f>
+          <t>Capacity: Target utilization at peak</t>
+        </is>
+      </c>
+      <c r="C27" s="50" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D27" s="51" t="n"/>
+      <c r="E27" s="27">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D27),D27&gt;=0.05,D27&lt;=1),D27,C27),C27)</f>
         <v/>
       </c>
       <c r="F27" s="3">
-        <f>IFERROR(IF(ISBLANK(D27),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D27),"Ignored: error value",IF(NOT(ISNUMBER(D27)),"Ignored: not a number",IF(OR(D27&lt;1,D27&gt;20),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <f>IFERROR(IF(ISBLANK(D27),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D27),"Ignored: error value",IF(NOT(ISNUMBER(D27)),"Ignored: not a number",IF(OR(D27&lt;0.05,D27&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
         <v/>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>1 to 20</t>
+          <t>0.05 to 1</t>
         </is>
       </c>
       <c r="H27" s="18" t="n"/>
@@ -10416,32 +10416,122 @@
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
+          <t>capacity.reserved_rate</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Capacity: Reserved rate ($ / GPU-hour)</t>
+        </is>
+      </c>
+      <c r="C28" s="56" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="D28" s="57" t="n"/>
+      <c r="E28" s="58">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D28),D28&gt;=0,D28&lt;=100),D28,C28),C28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="3">
+        <f>IFERROR(IF(ISBLANK(D28),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D28),"Ignored: error value",IF(NOT(ISNUMBER(D28)),"Ignored: not a number",IF(OR(D28&lt;0,D28&gt;100),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <v/>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>0 to 100</t>
+        </is>
+      </c>
+      <c r="H28" s="18" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>capacity.on_demand_rate</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Capacity: On-demand rate ($ / GPU-hour)</t>
+        </is>
+      </c>
+      <c r="C29" s="56" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="D29" s="57" t="n"/>
+      <c r="E29" s="58">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D29),D29&gt;=0,D29&lt;=100),D29,C29),C29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="3">
+        <f>IFERROR(IF(ISBLANK(D29),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D29),"Ignored: error value",IF(NOT(ISNUMBER(D29)),"Ignored: not a number",IF(OR(D29&lt;0,D29&gt;100),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <v/>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>0 to 100</t>
+        </is>
+      </c>
+      <c r="H29" s="18" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>capacity.peak_ratio_override</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Capacity: Peak hour / average (override if no hourly data)</t>
+        </is>
+      </c>
+      <c r="C30" s="47" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="D30" s="48" t="n"/>
+      <c r="E30" s="49">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D30),D30&gt;=1,D30&lt;=20),D30,C30),C30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="3">
+        <f>IFERROR(IF(ISBLANK(D30),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D30),"Ignored: error value",IF(NOT(ISNUMBER(D30)),"Ignored: not a number",IF(OR(D30&lt;1,D30&gt;20),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <v/>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>1 to 20</t>
+        </is>
+      </c>
+      <c r="H30" s="18" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
           <t>capacity.base_ratio_override</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Capacity: Quietest hour / average (override if no hourly data)</t>
         </is>
       </c>
-      <c r="C28" s="47" t="n">
+      <c r="C31" s="47" t="n">
         <v>0.55</v>
       </c>
-      <c r="D28" s="48" t="n"/>
-      <c r="E28" s="49">
-        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D28),D28&gt;=0,D28&lt;=1),D28,C28),C28)</f>
-        <v/>
-      </c>
-      <c r="F28" s="3">
-        <f>IFERROR(IF(ISBLANK(D28),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D28),"Ignored: error value",IF(NOT(ISNUMBER(D28)),"Ignored: not a number",IF(OR(D28&lt;0,D28&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
-        <v/>
-      </c>
-      <c r="G28" s="7" t="inlineStr">
+      <c r="D31" s="48" t="n"/>
+      <c r="E31" s="49">
+        <f>IFERROR(IF(AND(Overrides!$C$4="ON",ISNUMBER(D31),D31&gt;=0,D31&lt;=1),D31,C31),C31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="3">
+        <f>IFERROR(IF(ISBLANK(D31),"",IF(Overrides!$C$4&lt;&gt;"ON","Switch OFF",IF(ISERROR(D31),"Ignored: error value",IF(NOT(ISNUMBER(D31)),"Ignored: not a number",IF(OR(D31&lt;0,D31&gt;1),"Ignored: outside range","Applied"))))),"Ignored: error value")</f>
+        <v/>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>0 to 1</t>
         </is>
       </c>
-      <c r="H28" s="18" t="n"/>
+      <c r="H31" s="18" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -11083,7 +11173,7 @@
       <formula>$C$4="ON"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="25">
+  <dataValidations count="28">
     <dataValidation sqref="C4" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="ON or OFF" error="Choose ON or OFF." type="list">
       <formula1>"ON,OFF"</formula1>
     </dataValidation>
@@ -11134,51 +11224,63 @@
       <formula1>-0.5</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="D17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from -0.5 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D17" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 0.5, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>0.5</formula2>
+    </dataValidation>
+    <dataValidation sqref="D18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 0.5, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>0.5</formula2>
+    </dataValidation>
+    <dataValidation sqref="D19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 0.5, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+      <formula1>0</formula1>
+      <formula2>0.5</formula2>
+    </dataValidation>
+    <dataValidation sqref="D20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from -0.5 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>-0.5</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="D18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 2, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D21" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 2, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>2</formula2>
     </dataValidation>
-    <dataValidation sqref="D19" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 1 to 365, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 1 to 365, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>1</formula1>
       <formula2>365</formula2>
     </dataValidation>
-    <dataValidation sqref="D20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="D21" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="D22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D25" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="D23" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 1 to 1e+07, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 1 to 1e+07, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>1</formula1>
       <formula2>10000000</formula2>
     </dataValidation>
-    <dataValidation sqref="D24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0.05 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0.05 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>0.05</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation sqref="D25" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 100, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D28" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 100, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="D26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 100, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D29" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 100, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>
-    <dataValidation sqref="D27" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 1 to 20, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 1 to 20, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>1</formula1>
       <formula2>20</formula2>
     </dataValidation>
-    <dataValidation sqref="D28" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
+    <dataValidation sqref="D31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Outside the allowed range" error="Enter a number from 0 to 1, or leave blank to use the model value." type="decimal" errorStyle="stop" operator="between">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -29045,7 +29147,7 @@
         </is>
       </c>
       <c r="B7" s="11">
-        <f>Overrides!$E$17</f>
+        <f>Overrides!$E$20</f>
         <v/>
       </c>
       <c r="C7" s="25">
@@ -29117,7 +29219,7 @@
         </is>
       </c>
       <c r="C10" s="35">
-        <f>Overrides!$E$18</f>
+        <f>Overrides!$E$21</f>
         <v/>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -29177,7 +29279,7 @@
         </is>
       </c>
       <c r="C13" s="12">
-        <f>Overrides!$E$19</f>
+        <f>Overrides!$E$22</f>
         <v/>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -29193,7 +29295,7 @@
         </is>
       </c>
       <c r="C14" s="13">
-        <f>Overrides!$E$20</f>
+        <f>Overrides!$E$23</f>
         <v/>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -29209,7 +29311,7 @@
         </is>
       </c>
       <c r="C15" s="13">
-        <f>Overrides!$E$21</f>
+        <f>Overrides!$E$24</f>
         <v/>
       </c>
       <c r="E15" s="7" t="inlineStr"/>
@@ -29230,7 +29332,30 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Self-serve tokens lost to competitors, per month</t>
+        </is>
+      </c>
+      <c r="B17" s="11">
+        <f>Overrides!$E$17</f>
+        <v/>
+      </c>
+      <c r="C17" s="37">
+        <f>Overrides!$E$18</f>
+        <v/>
+      </c>
+      <c r="D17" s="11">
+        <f>Overrides!$E$19</f>
+        <v/>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Rival decision APIs (OpenAI Decisions API, AWS Strands Decider). Compounds monthly.</t>
+        </is>
+      </c>
+    </row>
     <row r="18"/>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -32603,15 +32728,15 @@
         </is>
       </c>
       <c r="B111" s="24">
-        <f>SUM(P51,O52,N53,M54,L55,K56,J57,I58,H59,G60,F61,E62,D63)+$C$16*$B$6^1</f>
+        <f>(SUM(P51,O52,N53,M54,L55,K56,J57,I58,H59,G60,F61,E62,D63)+$C$16*$B$6^1)*(1-$B$17)^1</f>
         <v/>
       </c>
       <c r="C111" s="24">
-        <f>SUM(Q51,P52,O53,N54,M55,L56,K57,J58,I59,H60,G61,F62,E63,D64)+$C$16*$B$6^2</f>
+        <f>(SUM(Q51,P52,O53,N54,M55,L56,K57,J58,I59,H60,G61,F62,E63,D64)+$C$16*$B$6^2)*(1-$B$17)^2</f>
         <v/>
       </c>
       <c r="D111" s="24">
-        <f>SUM(R51,Q52,P53,O54,N55,M56,L57,K58,J59,I60,H61,G62,F63,E64,D65)+$C$16*$B$6^3</f>
+        <f>(SUM(R51,Q52,P53,O54,N55,M56,L57,K58,J59,I60,H61,G62,F63,E64,D65)+$C$16*$B$6^3)*(1-$B$17)^3</f>
         <v/>
       </c>
     </row>
@@ -32622,15 +32747,15 @@
         </is>
       </c>
       <c r="B112" s="24">
-        <f>SUM(P71,O72,N73,M74,L75,K76,J77,I78,H79,G80,F81,E82,D83)+$C$16*$C$6^1</f>
+        <f>(SUM(P71,O72,N73,M74,L75,K76,J77,I78,H79,G80,F81,E82,D83)+$C$16*$C$6^1)*(1-$C$17)^1</f>
         <v/>
       </c>
       <c r="C112" s="24">
-        <f>SUM(Q71,P72,O73,N74,M75,L76,K77,J78,I79,H80,G81,F82,E83,D84)+$C$16*$C$6^2</f>
+        <f>(SUM(Q71,P72,O73,N74,M75,L76,K77,J78,I79,H80,G81,F82,E83,D84)+$C$16*$C$6^2)*(1-$C$17)^2</f>
         <v/>
       </c>
       <c r="D112" s="24">
-        <f>SUM(R71,Q72,P73,O74,N75,M76,L77,K78,J79,I80,H81,G82,F83,E84,D85)+$C$16*$C$6^3</f>
+        <f>(SUM(R71,Q72,P73,O74,N75,M76,L77,K78,J79,I80,H81,G82,F83,E84,D85)+$C$16*$C$6^3)*(1-$C$17)^3</f>
         <v/>
       </c>
     </row>
@@ -32641,15 +32766,15 @@
         </is>
       </c>
       <c r="B113" s="24">
-        <f>SUM(P91,O92,N93,M94,L95,K96,J97,I98,H99,G100,F101,E102,D103)+$C$16*$D$6^1</f>
+        <f>(SUM(P91,O92,N93,M94,L95,K96,J97,I98,H99,G100,F101,E102,D103)+$C$16*$D$6^1)*(1-$D$17)^1</f>
         <v/>
       </c>
       <c r="C113" s="24">
-        <f>SUM(Q91,P92,O93,N94,M95,L96,K97,J98,I99,H100,G101,F102,E103,D104)+$C$16*$D$6^2</f>
+        <f>(SUM(Q91,P92,O93,N94,M95,L96,K97,J98,I99,H100,G101,F102,E103,D104)+$C$16*$D$6^2)*(1-$D$17)^2</f>
         <v/>
       </c>
       <c r="D113" s="24">
-        <f>SUM(R91,Q92,P93,O94,N95,M96,L97,K98,J99,I100,H101,G102,F103,E104,D105)+$C$16*$D$6^3</f>
+        <f>(SUM(R91,Q92,P93,O94,N95,M96,L97,K98,J99,I100,H101,G102,F103,E104,D105)+$C$16*$D$6^3)*(1-$D$17)^3</f>
         <v/>
       </c>
     </row>

</xml_diff>